<commit_message>
Antenna Tuner Instructions Update
Antenna Tuner Instructions Update
</commit_message>
<xml_diff>
--- a/K9HZ_LPF_Module/K9HZ_LPF_BOMs/K9HZ_LPF-TR Carrier_Board_BOM_V2.00_01-10-24.xlsx
+++ b/K9HZ_LPF_Module/K9HZ_LPF_BOMs/K9HZ_LPF-TR Carrier_Board_BOM_V2.00_01-10-24.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dad\Documents\GitHub\K9HZ\K9HZ_LPF_Module\K9HZ_LPF_BOMs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bill\Documents\GitHub\K9HZ\K9HZ_LPF_Module\K9HZ_LPF_BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10D1207-5D5B-476A-8D46-7FB7237AA4E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD941001-8832-4351-94F5-E38E3BE8589F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T41-WJS-10-band-LPF-TR-carrier" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Quantity</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Comments</t>
   </si>
   <si>
-    <t>0.1uF 50V</t>
-  </si>
-  <si>
     <t>C1, C2</t>
   </si>
   <si>
@@ -76,9 +73,6 @@
     <t>K1, K2</t>
   </si>
   <si>
-    <t>Surplus</t>
-  </si>
-  <si>
     <t>BS170 FET</t>
   </si>
   <si>
@@ -106,9 +100,6 @@
     <t>71-RCP1206W50R0GEB</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>J1, J2</t>
   </si>
   <si>
@@ -116,13 +107,19 @@
   </si>
   <si>
     <t>SMA Female PCB Mount Connector</t>
+  </si>
+  <si>
+    <t>0.1uF 50V SMD 1206</t>
+  </si>
+  <si>
+    <t>Surplus (Aliexpress)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,6 +253,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -599,14 +608,18 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -962,27 +975,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.90625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="33.36328125" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.453125" customWidth="1"/>
-    <col min="6" max="6" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="33.33203125" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
@@ -997,122 +1010,141 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
+      <c r="D3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>4</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>1</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>1</v>
       </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="1">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="B9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="1">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="D9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>28</v>
-      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>